<commit_message>
feat(database): import Mon/Thu afternoon lower-grade remedial classes (學2甲, 學2乙) and update Grade 2 students
</commit_message>
<xml_diff>
--- a/public/templates/清水國小全校師生名冊_匯入範本.xlsx
+++ b/public/templates/清水國小全校師生名冊_匯入範本.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2145"/>
+  <dimension ref="A1:I2156"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -7990,13 +7990,13 @@
         <v>05號</v>
       </c>
       <c r="D262" t="str">
-        <v>葉宥廷</v>
+        <v>陳育豪</v>
       </c>
       <c r="E262" t="str">
-        <v>葉宥廷家長</v>
+        <v>陳育豪家長</v>
       </c>
       <c r="F262" t="str">
-        <v>0981-100-448</v>
+        <v>0929880813</v>
       </c>
       <c r="G262" t="str">
         <v>張老師</v>
@@ -8570,13 +8570,13 @@
         <v>25號</v>
       </c>
       <c r="D282" t="str">
-        <v>鄭宥廷</v>
+        <v>黃馨苓</v>
       </c>
       <c r="E282" t="str">
-        <v>鄭宥廷家長</v>
+        <v>黃馨苓家長</v>
       </c>
       <c r="F282" t="str">
-        <v>0925-720-609</v>
+        <v>0931897858</v>
       </c>
       <c r="G282" t="str">
         <v>張老師</v>
@@ -9063,13 +9063,13 @@
         <v>16號</v>
       </c>
       <c r="D299" t="str">
-        <v>高芷晴</v>
+        <v>張絃霏</v>
       </c>
       <c r="E299" t="str">
-        <v>高芷晴家長</v>
+        <v>張絃霏家長</v>
       </c>
       <c r="F299" t="str">
-        <v>0917-348-611</v>
+        <v>0918209668</v>
       </c>
       <c r="G299" t="str">
         <v>吳老師</v>
@@ -10368,13 +10368,13 @@
         <v>06號</v>
       </c>
       <c r="D344" t="str">
-        <v>洪宥辰</v>
+        <v>施文凱</v>
       </c>
       <c r="E344" t="str">
-        <v>洪宥辰家長</v>
+        <v>施文凱家長</v>
       </c>
       <c r="F344" t="str">
-        <v>0989-844-299</v>
+        <v>0986494806</v>
       </c>
       <c r="G344" t="str">
         <v>謝老師</v>
@@ -11151,13 +11151,13 @@
         <v>06號</v>
       </c>
       <c r="D371" t="str">
-        <v>許子軒</v>
+        <v>傅昱霖</v>
       </c>
       <c r="E371" t="str">
-        <v>許子軒家長</v>
+        <v>傅昱霖家長</v>
       </c>
       <c r="F371" t="str">
-        <v>0953-782-831</v>
+        <v>0960741037</v>
       </c>
       <c r="G371" t="str">
         <v>邱老師</v>
@@ -13500,13 +13500,13 @@
         <v>10號</v>
       </c>
       <c r="D452" t="str">
-        <v>陳若瑄</v>
+        <v>劉羽洋</v>
       </c>
       <c r="E452" t="str">
-        <v>陳若瑄家長</v>
+        <v>劉羽洋家長</v>
       </c>
       <c r="F452" t="str">
-        <v>0944-596-629</v>
+        <v>0928424077</v>
       </c>
       <c r="G452" t="str">
         <v>江老師</v>
@@ -13529,13 +13529,13 @@
         <v>11號</v>
       </c>
       <c r="D453" t="str">
-        <v>黃浩宇</v>
+        <v>張耿愷</v>
       </c>
       <c r="E453" t="str">
-        <v>黃浩宇家長</v>
+        <v>張耿愷家長</v>
       </c>
       <c r="F453" t="str">
-        <v>0961-627-682</v>
+        <v>0911587027</v>
       </c>
       <c r="G453" t="str">
         <v>江老師</v>
@@ -14602,13 +14602,13 @@
         <v>20號</v>
       </c>
       <c r="D490" t="str">
-        <v>楊宥辰</v>
+        <v>許美梅</v>
       </c>
       <c r="E490" t="str">
-        <v>楊宥辰家長</v>
+        <v>許美梅家長</v>
       </c>
       <c r="F490" t="str">
-        <v>0996-875-845</v>
+        <v>0970055872</v>
       </c>
       <c r="G490" t="str">
         <v>羅老師</v>
@@ -15269,13 +15269,13 @@
         <v>17號</v>
       </c>
       <c r="D513" t="str">
-        <v>黃柏翰</v>
+        <v>陳秀妍</v>
       </c>
       <c r="E513" t="str">
-        <v>黃柏翰家長</v>
+        <v>陳秀妍家長</v>
       </c>
       <c r="F513" t="str">
-        <v>0991-689-266</v>
+        <v>0925705178</v>
       </c>
       <c r="G513" t="str">
         <v>林老師</v>
@@ -15472,13 +15472,13 @@
         <v>24號</v>
       </c>
       <c r="D520" t="str">
-        <v>楊浩宇</v>
+        <v>江羽恩</v>
       </c>
       <c r="E520" t="str">
-        <v>楊浩宇家長</v>
+        <v>江羽恩家長</v>
       </c>
       <c r="F520" t="str">
-        <v>0912-906-637</v>
+        <v>0905030069</v>
       </c>
       <c r="G520" t="str">
         <v>林老師</v>
@@ -62615,9 +62615,328 @@
         <v>在籍</v>
       </c>
     </row>
+    <row r="2146">
+      <c r="A2146" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2146" t="str">
+        <v>學2甲</v>
+      </c>
+      <c r="C2146" t="str">
+        <v>01號</v>
+      </c>
+      <c r="D2146" t="str">
+        <v>陳育豪</v>
+      </c>
+      <c r="E2146" t="str">
+        <v>陳育豪家長</v>
+      </c>
+      <c r="F2146" t="str">
+        <v>0929880813</v>
+      </c>
+      <c r="G2146" t="str">
+        <v>學2甲輔導師</v>
+      </c>
+      <c r="H2146" t="str">
+        <v>0966-333-001</v>
+      </c>
+      <c r="I2146" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2147" t="str">
+        <v>學2甲</v>
+      </c>
+      <c r="C2147" t="str">
+        <v>02號</v>
+      </c>
+      <c r="D2147" t="str">
+        <v>黃馨苓</v>
+      </c>
+      <c r="E2147" t="str">
+        <v>黃馨苓家長</v>
+      </c>
+      <c r="F2147" t="str">
+        <v>0931897858</v>
+      </c>
+      <c r="G2147" t="str">
+        <v>學2甲輔導師</v>
+      </c>
+      <c r="H2147" t="str">
+        <v>0966-333-001</v>
+      </c>
+      <c r="I2147" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2148" t="str">
+        <v>學2甲</v>
+      </c>
+      <c r="C2148" t="str">
+        <v>03號</v>
+      </c>
+      <c r="D2148" t="str">
+        <v>張絃霏</v>
+      </c>
+      <c r="E2148" t="str">
+        <v>張絃霏家長</v>
+      </c>
+      <c r="F2148" t="str">
+        <v>0918209668</v>
+      </c>
+      <c r="G2148" t="str">
+        <v>學2甲輔導師</v>
+      </c>
+      <c r="H2148" t="str">
+        <v>0966-333-001</v>
+      </c>
+      <c r="I2148" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2149" t="str">
+        <v>學2甲</v>
+      </c>
+      <c r="C2149" t="str">
+        <v>04號</v>
+      </c>
+      <c r="D2149" t="str">
+        <v>施文凱</v>
+      </c>
+      <c r="E2149" t="str">
+        <v>施文凱家長</v>
+      </c>
+      <c r="F2149" t="str">
+        <v>0986494806</v>
+      </c>
+      <c r="G2149" t="str">
+        <v>學2甲輔導師</v>
+      </c>
+      <c r="H2149" t="str">
+        <v>0966-333-001</v>
+      </c>
+      <c r="I2149" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2150" t="str">
+        <v>學2甲</v>
+      </c>
+      <c r="C2150" t="str">
+        <v>05號</v>
+      </c>
+      <c r="D2150" t="str">
+        <v>傅昱霖</v>
+      </c>
+      <c r="E2150" t="str">
+        <v>傅昱霖家長</v>
+      </c>
+      <c r="F2150" t="str">
+        <v>0960741037</v>
+      </c>
+      <c r="G2150" t="str">
+        <v>學2甲輔導師</v>
+      </c>
+      <c r="H2150" t="str">
+        <v>0966-333-001</v>
+      </c>
+      <c r="I2150" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2151" t="str">
+        <v>學2乙</v>
+      </c>
+      <c r="C2151" t="str">
+        <v>01號</v>
+      </c>
+      <c r="D2151" t="str">
+        <v>劉羽洋</v>
+      </c>
+      <c r="E2151" t="str">
+        <v>劉羽洋家長</v>
+      </c>
+      <c r="F2151" t="str">
+        <v>0928424077</v>
+      </c>
+      <c r="G2151" t="str">
+        <v>學2乙輔導師</v>
+      </c>
+      <c r="H2151" t="str">
+        <v>0966-333-002</v>
+      </c>
+      <c r="I2151" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2152" t="str">
+        <v>學2乙</v>
+      </c>
+      <c r="C2152" t="str">
+        <v>02號</v>
+      </c>
+      <c r="D2152" t="str">
+        <v>張耿愷</v>
+      </c>
+      <c r="E2152" t="str">
+        <v>張耿愷家長</v>
+      </c>
+      <c r="F2152" t="str">
+        <v>0911587027</v>
+      </c>
+      <c r="G2152" t="str">
+        <v>學2乙輔導師</v>
+      </c>
+      <c r="H2152" t="str">
+        <v>0966-333-002</v>
+      </c>
+      <c r="I2152" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2153" t="str">
+        <v>學2乙</v>
+      </c>
+      <c r="C2153" t="str">
+        <v>03號</v>
+      </c>
+      <c r="D2153" t="str">
+        <v>許美梅</v>
+      </c>
+      <c r="E2153" t="str">
+        <v>許美梅家長</v>
+      </c>
+      <c r="F2153" t="str">
+        <v>0970055872</v>
+      </c>
+      <c r="G2153" t="str">
+        <v>學2乙輔導師</v>
+      </c>
+      <c r="H2153" t="str">
+        <v>0966-333-002</v>
+      </c>
+      <c r="I2153" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2154" t="str">
+        <v>學2乙</v>
+      </c>
+      <c r="C2154" t="str">
+        <v>04號</v>
+      </c>
+      <c r="D2154" t="str">
+        <v>廖怡靚</v>
+      </c>
+      <c r="E2154" t="str">
+        <v>廖怡靚家長</v>
+      </c>
+      <c r="F2154" t="str">
+        <v>0922604000</v>
+      </c>
+      <c r="G2154" t="str">
+        <v>學2乙輔導師</v>
+      </c>
+      <c r="H2154" t="str">
+        <v>0966-333-002</v>
+      </c>
+      <c r="I2154" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2155" t="str">
+        <v>學2乙</v>
+      </c>
+      <c r="C2155" t="str">
+        <v>05號</v>
+      </c>
+      <c r="D2155" t="str">
+        <v>陳秀妍</v>
+      </c>
+      <c r="E2155" t="str">
+        <v>陳秀妍家長</v>
+      </c>
+      <c r="F2155" t="str">
+        <v>0925705178</v>
+      </c>
+      <c r="G2155" t="str">
+        <v>學2乙輔導師</v>
+      </c>
+      <c r="H2155" t="str">
+        <v>0966-333-002</v>
+      </c>
+      <c r="I2155" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" t="str">
+        <v>學習扶助班</v>
+      </c>
+      <c r="B2156" t="str">
+        <v>學2乙</v>
+      </c>
+      <c r="C2156" t="str">
+        <v>06號</v>
+      </c>
+      <c r="D2156" t="str">
+        <v>江羽恩</v>
+      </c>
+      <c r="E2156" t="str">
+        <v>江羽恩家長</v>
+      </c>
+      <c r="F2156" t="str">
+        <v>0905030069</v>
+      </c>
+      <c r="G2156" t="str">
+        <v>學2乙輔導師</v>
+      </c>
+      <c r="H2156" t="str">
+        <v>0966-333-002</v>
+      </c>
+      <c r="I2156" t="str">
+        <v>在籍</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2145"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2156"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>